<commit_message>
Feat: Adicionando novos passos e atualizações de desempenho
</commit_message>
<xml_diff>
--- a/Provisionamento/provisionamento.xlsx
+++ b/Provisionamento/provisionamento.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="164011"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\espro.mvsilva\OneDrive - Azul Linhas Aéreas Brasileiras\Área de Trabalho\Python automação\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\espro.mvsilva\OneDrive - Azul Linhas Aéreas Brasileiras\Área de Trabalho\Python automação\Provisionamento\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="11">
   <si>
     <t>ID Processo</t>
   </si>
@@ -38,34 +38,25 @@
     <t>Processo</t>
   </si>
   <si>
-    <t>FISCALIZAÇÃO</t>
-  </si>
-  <si>
-    <t>REBHKNXC5J1XP4</t>
-  </si>
-  <si>
-    <t>IGU</t>
-  </si>
-  <si>
-    <t>REBHKNXMHSY0B3</t>
-  </si>
-  <si>
-    <t>REBHKNXMGZX9G1</t>
-  </si>
-  <si>
-    <t>MGF</t>
-  </si>
-  <si>
-    <t>REBHKNXC5602C7</t>
-  </si>
-  <si>
-    <t>REBHKNXMG78H3F</t>
-  </si>
-  <si>
-    <t>LDB</t>
-  </si>
-  <si>
-    <t>REBHKNXC4SH7XY</t>
+    <t>23.375.153-0</t>
+  </si>
+  <si>
+    <t>REC</t>
+  </si>
+  <si>
+    <t>Auto de Infração</t>
+  </si>
+  <si>
+    <t>23.375.078-9</t>
+  </si>
+  <si>
+    <t>PNZ</t>
+  </si>
+  <si>
+    <t>23.385.945-4</t>
+  </si>
+  <si>
+    <t>THE</t>
   </si>
 </sst>
 </file>
@@ -151,16 +142,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -448,7 +436,7 @@
     <col min="1" max="1" width="13.5703125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="23.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="34.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.5703125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="15.75" x14ac:dyDescent="0.25">
@@ -467,87 +455,63 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
-        <v>988256</v>
+        <v>1009031</v>
       </c>
       <c r="B2" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>6</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
-        <v>988258</v>
+        <v>1009032</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>7</v>
       </c>
       <c r="C3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>6</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
-        <v>988260</v>
-      </c>
-      <c r="B4" s="3" t="s">
-        <v>8</v>
+        <v>1009034</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>9</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A5" s="2">
-        <v>988262</v>
-      </c>
-      <c r="B5" s="2" t="s">
-        <v>10</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="D5" s="2" t="s">
-        <v>4</v>
-      </c>
+      <c r="A5" s="2"/>
+      <c r="B5" s="2"/>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A6" s="2">
-        <v>988264</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>4</v>
-      </c>
+      <c r="A6" s="2"/>
+      <c r="B6" s="2"/>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A7" s="2">
-        <v>988265</v>
-      </c>
-      <c r="B7" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="D7" s="2" t="s">
-        <v>4</v>
-      </c>
+      <c r="A7" s="2"/>
+      <c r="B7" s="2"/>
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
@@ -555,23 +519,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="cdc37f11-6699-4390-935e-7d00f6a9cb17" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010040810410046D4846AFC1D9D1724EAE0C" ma:contentTypeVersion="10" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="3cf92e38dbd5ca6e29a3dbc90f9259c3">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="cdc37f11-6699-4390-935e-7d00f6a9cb17" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3b7840fd93bba6919c464d2db268669e" ns3:_="">
     <xsd:import namespace="cdc37f11-6699-4390-935e-7d00f6a9cb17"/>
@@ -753,31 +700,24 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="cdc37f11-6699-4390-935e-7d00f6a9cb17" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E5CBD717-E7CA-471D-A675-1E703ACDF3D5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="cdc37f11-6699-4390-935e-7d00f6a9cb17"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7D2E150F-7C48-466A-AA6B-C8C58D0A952D}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9964EC62-F762-492F-9669-9C56E6C51FCE}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -793,4 +733,28 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7D2E150F-7C48-466A-AA6B-C8C58D0A952D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E5CBD717-E7CA-471D-A675-1E703ACDF3D5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="cdc37f11-6699-4390-935e-7d00f6a9cb17"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>